<commit_message>
Add scheduled Higgsfield article and plan
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -1366,7 +1366,7 @@
     <row r="4" ht="21.75" customHeight="1" s="115">
       <c r="B4" s="117" t="inlineStr">
         <is>
-          <t>Agentic AI &amp; Claude AI · 20 planned posts · Daily cadence from Apr 10</t>
+          <t>Agentic AI, Claude AI, and Higgsfield · 27 planned posts · Daily cadence through Apr 30</t>
         </is>
       </c>
     </row>
@@ -1385,15 +1385,11 @@
           <t>24</t>
         </is>
       </c>
-      <c r="C8" s="120" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D8" s="121" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C8" s="120" t="n">
+        <v>27</v>
+      </c>
+      <c r="D8" s="121" t="n">
+        <v>4</v>
       </c>
       <c r="E8" s="122" t="inlineStr">
         <is>
@@ -1427,7 +1423,7 @@
       <c r="D9" s="125" t="inlineStr">
         <is>
           <t>Tuần theo lịch mới
-(Apr 6 – Apr 23)</t>
+(Apr 6 – Apr 30)</t>
         </is>
       </c>
       <c r="E9" s="126" t="inlineStr">
@@ -1695,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:H24"/>
+  <dimension ref="B2:H34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -1711,7 +1707,7 @@
     <row r="2" ht="39.75" customHeight="1" s="115">
       <c r="B2" s="147" t="inlineStr">
         <is>
-          <t>LỊCH XUẤT BẢN — DAILY CADENCE (April 6 – April 23, 2026)</t>
+          <t>LỊCH XUẤT BẢN — DAILY CADENCE (April 6 – April 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -1791,106 +1787,106 @@
       </c>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="115">
-      <c r="B6" s="156" t="n"/>
-      <c r="C6" s="157" t="inlineStr">
+      <c r="B6" s="149" t="n"/>
+      <c r="C6" s="150" t="inlineStr">
         <is>
           <t>T4, 08/04</t>
         </is>
       </c>
-      <c r="D6" s="158" t="inlineStr">
+      <c r="D6" s="151" t="inlineStr">
         <is>
           <t>C0 — AI Flywheel là gì? Cách dùng Agentic AI tạo vòng lặp tăng trưởng tự động</t>
         </is>
       </c>
-      <c r="E6" s="159" t="inlineStr">
+      <c r="E6" s="152" t="inlineStr">
         <is>
           <t>Cluster C · AI Flywheel</t>
         </is>
       </c>
-      <c r="F6" s="160" t="inlineStr">
+      <c r="F6" s="153" t="inlineStr">
         <is>
           <t>Pillar (~3,000 từ)</t>
         </is>
       </c>
-      <c r="G6" s="161" t="inlineStr">
+      <c r="G6" s="154" t="inlineStr">
         <is>
           <t>ToF/MoF</t>
         </is>
       </c>
-      <c r="H6" s="162" t="inlineStr">
+      <c r="H6" s="155" t="inlineStr">
         <is>
           <t>🏷 Brand</t>
         </is>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1" s="115">
-      <c r="B7" s="163" t="n"/>
-      <c r="C7" s="164" t="inlineStr">
+      <c r="B7" s="149" t="n"/>
+      <c r="C7" s="150" t="inlineStr">
         <is>
           <t>T5, 09/04</t>
         </is>
       </c>
-      <c r="D7" s="165" t="inlineStr">
+      <c r="D7" s="151" t="inlineStr">
         <is>
           <t>D3 — Khi AI bị rò rỉ source code: Bài học từ Claude Code leaked 2.4M views</t>
         </is>
       </c>
-      <c r="E7" s="166" t="inlineStr">
+      <c r="E7" s="152" t="inlineStr">
         <is>
           <t>Cluster D · News</t>
         </is>
       </c>
-      <c r="F7" s="167" t="inlineStr">
+      <c r="F7" s="153" t="inlineStr">
         <is>
           <t>Newsjack (~1,000 từ)</t>
         </is>
       </c>
-      <c r="G7" s="168" t="inlineStr">
+      <c r="G7" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H7" s="169" t="inlineStr">
+      <c r="H7" s="155" t="inlineStr">
         <is>
           <t>🚀 Viral</t>
         </is>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1" s="115">
-      <c r="B8" s="170" t="n"/>
-      <c r="C8" s="171" t="inlineStr">
+      <c r="B8" s="149" t="n"/>
+      <c r="C8" s="150" t="inlineStr">
         <is>
           <t>T5, 09/04</t>
         </is>
       </c>
-      <c r="D8" s="172" t="inlineStr">
+      <c r="D8" s="151" t="inlineStr">
         <is>
           <t>B0 — Hướng dẫn sử dụng Claude AI toàn tập — từ cơ bản đến nâng cao 2026</t>
         </is>
       </c>
-      <c r="E8" s="173" t="inlineStr">
+      <c r="E8" s="152" t="inlineStr">
         <is>
           <t>Cluster B · Claude AI</t>
         </is>
       </c>
-      <c r="F8" s="174" t="inlineStr">
+      <c r="F8" s="153" t="inlineStr">
         <is>
           <t>Pillar (~3,500 từ)</t>
         </is>
       </c>
-      <c r="G8" s="175" t="inlineStr">
+      <c r="G8" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H8" s="176" t="inlineStr">
+      <c r="H8" s="155" t="inlineStr">
         <is>
           <t>🔥 Hot</t>
         </is>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1" s="115">
-      <c r="B9" s="177" t="n"/>
+      <c r="B9" s="149" t="n"/>
       <c r="C9" s="150" t="inlineStr">
         <is>
           <t>T6, 10/04</t>
@@ -1911,7 +1907,7 @@
           <t>Case Study (~2,200 từ)</t>
         </is>
       </c>
-      <c r="G9" s="155" t="inlineStr">
+      <c r="G9" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
@@ -1923,138 +1919,138 @@
       </c>
     </row>
     <row r="10" ht="31.5" customHeight="1" s="115">
-      <c r="B10" s="163" t="n"/>
-      <c r="C10" s="164" t="inlineStr">
+      <c r="B10" s="149" t="n"/>
+      <c r="C10" s="150" t="inlineStr">
         <is>
           <t>T7, 11/04</t>
         </is>
       </c>
-      <c r="D10" s="165" t="inlineStr">
+      <c r="D10" s="151" t="inlineStr">
         <is>
           <t>D1 — Claude Mythos, AGI mới và Claude Code Update: Điều gì đang xảy ra với AI tháng này?</t>
         </is>
       </c>
-      <c r="E10" s="166" t="inlineStr">
+      <c r="E10" s="152" t="inlineStr">
         <is>
           <t>Cluster D · News</t>
         </is>
       </c>
-      <c r="F10" s="167" t="inlineStr">
+      <c r="F10" s="153" t="inlineStr">
         <is>
           <t>News Roundup (~1,200 từ)</t>
         </is>
       </c>
-      <c r="G10" s="168" t="inlineStr">
+      <c r="G10" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H10" s="169" t="inlineStr">
+      <c r="H10" s="155" t="inlineStr">
         <is>
           <t>📰 News</t>
         </is>
       </c>
     </row>
     <row r="11" ht="31.5" customHeight="1" s="115">
-      <c r="B11" s="178" t="n"/>
-      <c r="C11" s="157" t="inlineStr">
+      <c r="B11" s="149" t="n"/>
+      <c r="C11" s="150" t="inlineStr">
         <is>
           <t>CN, 12/04</t>
         </is>
       </c>
-      <c r="D11" s="158" t="inlineStr">
+      <c r="D11" s="151" t="inlineStr">
         <is>
           <t>C1 — 5 cách kiếm tiền với Agentic AI năm 2026 — không ai làm (mà nên làm ngay)</t>
         </is>
       </c>
-      <c r="E11" s="159" t="inlineStr">
+      <c r="E11" s="152" t="inlineStr">
         <is>
           <t>Cluster C · AI Flywheel</t>
         </is>
       </c>
-      <c r="F11" s="160" t="inlineStr">
+      <c r="F11" s="153" t="inlineStr">
         <is>
           <t>Case Study (~2,000 từ)</t>
         </is>
       </c>
-      <c r="G11" s="179" t="inlineStr">
+      <c r="G11" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
       </c>
-      <c r="H11" s="162" t="inlineStr">
+      <c r="H11" s="155" t="inlineStr">
         <is>
           <t>🔥 Hot</t>
         </is>
       </c>
     </row>
     <row r="12" ht="31.5" customHeight="1" s="115">
-      <c r="B12" s="180" t="inlineStr">
+      <c r="B12" s="149" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="C12" s="171" t="inlineStr">
+      <c r="C12" s="150" t="inlineStr">
         <is>
           <t>T2, 13/04</t>
         </is>
       </c>
-      <c r="D12" s="172" t="inlineStr">
+      <c r="D12" s="151" t="inlineStr">
+        <is>
+          <t>H1 — What Is Higgsfield AI? A Practical Guide for Creators</t>
+        </is>
+      </c>
+      <c r="E12" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F12" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G12" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H12" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="31.5" customHeight="1" s="115">
+      <c r="B13" s="149" t="n"/>
+      <c r="C13" s="150" t="inlineStr">
+        <is>
+          <t>T3, 14/04</t>
+        </is>
+      </c>
+      <c r="D13" s="151" t="inlineStr">
         <is>
           <t>B2 — Claude vs ChatGPT vs Gemini 2026: So sánh chi tiết — cái nào tốt hơn cho content?</t>
         </is>
       </c>
-      <c r="E12" s="173" t="inlineStr">
+      <c r="E13" s="152" t="inlineStr">
         <is>
           <t>Cluster B · Claude AI</t>
         </is>
       </c>
-      <c r="F12" s="174" t="inlineStr">
+      <c r="F13" s="153" t="inlineStr">
         <is>
           <t>So Sánh (~2,800 từ)</t>
         </is>
       </c>
-      <c r="G12" s="181" t="inlineStr">
+      <c r="G13" s="154" t="inlineStr">
         <is>
           <t>MoF/BoF</t>
         </is>
       </c>
-      <c r="H12" s="176" t="inlineStr">
+      <c r="H13" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="31.5" customHeight="1" s="115">
-      <c r="B13" s="182" t="n"/>
-      <c r="C13" s="183" t="inlineStr">
-        <is>
-          <t>T3, 14/04</t>
-        </is>
-      </c>
-      <c r="D13" s="184" t="inlineStr">
-        <is>
-          <t>A2 — AI Agent vs AI Assistant: Khác nhau thế nào và dùng cái nào cho phù hợp?</t>
-        </is>
-      </c>
-      <c r="E13" s="185" t="inlineStr">
-        <is>
-          <t>Cluster A · Agentic AI</t>
-        </is>
-      </c>
-      <c r="F13" s="186" t="inlineStr">
-        <is>
-          <t>So Sánh (~1,800 từ)</t>
-        </is>
-      </c>
-      <c r="G13" s="187" t="inlineStr">
-        <is>
-          <t>ToF</t>
-        </is>
-      </c>
-      <c r="H13" s="188" t="inlineStr">
-        <is>
-          <t>📌 Med</t>
         </is>
       </c>
     </row>
@@ -2067,309 +2063,548 @@
       </c>
       <c r="D14" s="151" t="inlineStr">
         <is>
+          <t>H2 — Higgsfield for Beginners: What to Test First</t>
+        </is>
+      </c>
+      <c r="E14" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F14" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~1,600 từ)</t>
+        </is>
+      </c>
+      <c r="G14" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H14" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="31.5" customHeight="1" s="115">
+      <c r="B15" s="149" t="n"/>
+      <c r="C15" s="150" t="inlineStr">
+        <is>
+          <t>T5, 16/04</t>
+        </is>
+      </c>
+      <c r="D15" s="151" t="inlineStr">
+        <is>
+          <t>A2 — AI Agent vs AI Assistant: Khác nhau thế nào và dùng cái nào cho phù hợp?</t>
+        </is>
+      </c>
+      <c r="E15" s="152" t="inlineStr">
+        <is>
+          <t>Cluster A · Agentic AI</t>
+        </is>
+      </c>
+      <c r="F15" s="153" t="inlineStr">
+        <is>
+          <t>So Sánh (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G15" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H15" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="31.5" customHeight="1" s="115">
+      <c r="B16" s="149" t="n"/>
+      <c r="C16" s="150" t="inlineStr">
+        <is>
+          <t>T6, 17/04</t>
+        </is>
+      </c>
+      <c r="D16" s="151" t="inlineStr">
+        <is>
+          <t>H3 — Best Use Cases for Higgsfield in Short-Form Content Workflows</t>
+        </is>
+      </c>
+      <c r="E16" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F16" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G16" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H16" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="31.5" customHeight="1" s="115">
+      <c r="B17" s="149" t="n"/>
+      <c r="C17" s="150" t="inlineStr">
+        <is>
+          <t>T7, 18/04</t>
+        </is>
+      </c>
+      <c r="D17" s="151" t="inlineStr">
+        <is>
           <t>A3 — Cách xây dựng AI Agent đầu tiên cho content marketing — không cần code</t>
         </is>
       </c>
-      <c r="E14" s="152" t="inlineStr">
+      <c r="E17" s="152" t="inlineStr">
         <is>
           <t>Cluster A · Agentic AI</t>
         </is>
       </c>
-      <c r="F14" s="153" t="inlineStr">
+      <c r="F17" s="153" t="inlineStr">
         <is>
           <t>How-to (~2,500 từ)</t>
         </is>
       </c>
-      <c r="G14" s="155" t="inlineStr">
+      <c r="G17" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
       </c>
-      <c r="H14" s="155" t="inlineStr">
+      <c r="H17" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="31.5" customHeight="1" s="115">
-      <c r="B15" s="180" t="n"/>
-      <c r="C15" s="171" t="inlineStr">
-        <is>
-          <t>T5, 16/04</t>
-        </is>
-      </c>
-      <c r="D15" s="172" t="inlineStr">
+    <row r="18" ht="31.5" customHeight="1" s="115">
+      <c r="B18" s="149" t="n"/>
+      <c r="C18" s="150" t="inlineStr">
+        <is>
+          <t>CN, 19/04</t>
+        </is>
+      </c>
+      <c r="D18" s="151" t="inlineStr">
+        <is>
+          <t>H4 — Higgsfield vs Runway: Which One Fits Faster Creator Workflows?</t>
+        </is>
+      </c>
+      <c r="E18" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F18" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G18" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H18" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="31.5" customHeight="1" s="115">
+      <c r="B19" s="149" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="C19" s="150" t="inlineStr">
+        <is>
+          <t>T2, 20/04</t>
+        </is>
+      </c>
+      <c r="D19" s="151" t="inlineStr">
         <is>
           <t>B3 — 10 prompt Claude AI tốt nhất cho content marketing — copy và dùng ngay</t>
         </is>
       </c>
-      <c r="E15" s="173" t="inlineStr">
+      <c r="E19" s="152" t="inlineStr">
         <is>
           <t>Cluster B · Claude AI</t>
         </is>
       </c>
-      <c r="F15" s="174" t="inlineStr">
+      <c r="F19" s="153" t="inlineStr">
         <is>
           <t>How-to (~1,800 từ)</t>
         </is>
       </c>
-      <c r="G15" s="181" t="inlineStr">
+      <c r="G19" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
       </c>
-      <c r="H15" s="176" t="inlineStr">
+      <c r="H19" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="31.5" customHeight="1" s="115">
-      <c r="B16" s="163" t="n"/>
-      <c r="C16" s="164" t="inlineStr">
-        <is>
-          <t>T6, 17/04</t>
-        </is>
-      </c>
-      <c r="D16" s="165" t="inlineStr">
+    <row r="20" ht="31.5" customHeight="1" s="115">
+      <c r="B20" s="149" t="n"/>
+      <c r="C20" s="150" t="inlineStr">
+        <is>
+          <t>T3, 21/04</t>
+        </is>
+      </c>
+      <c r="D20" s="151" t="inlineStr">
+        <is>
+          <t>H5 — Higgsfield Alternatives: When to Choose Another AI Visual Tool</t>
+        </is>
+      </c>
+      <c r="E20" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F20" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G20" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H20" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="31.5" customHeight="1" s="115">
+      <c r="B21" s="149" t="n"/>
+      <c r="C21" s="150" t="inlineStr">
+        <is>
+          <t>T4, 22/04</t>
+        </is>
+      </c>
+      <c r="D21" s="151" t="inlineStr">
         <is>
           <t>D2 — Qwen3 của Alibaba có thật sự nguy hiểm cho Anthropic? Phân tích kỹ thuật không hype</t>
         </is>
       </c>
-      <c r="E16" s="166" t="inlineStr">
+      <c r="E21" s="152" t="inlineStr">
         <is>
           <t>Cluster D · News</t>
         </is>
       </c>
-      <c r="F16" s="167" t="inlineStr">
+      <c r="F21" s="153" t="inlineStr">
         <is>
           <t>Analysis (~1,500 từ)</t>
         </is>
       </c>
-      <c r="G16" s="168" t="inlineStr">
+      <c r="G21" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H16" s="169" t="inlineStr">
+      <c r="H21" s="155" t="inlineStr">
         <is>
           <t>📰 News</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="31.5" customHeight="1" s="115">
-      <c r="B17" s="178" t="n"/>
-      <c r="C17" s="157" t="inlineStr">
-        <is>
-          <t>T7, 18/04</t>
-        </is>
-      </c>
-      <c r="D17" s="158" t="inlineStr">
+    <row r="22" ht="31.5" customHeight="1" s="115">
+      <c r="B22" s="149" t="n"/>
+      <c r="C22" s="150" t="inlineStr">
+        <is>
+          <t>T5, 23/04</t>
+        </is>
+      </c>
+      <c r="D22" s="151" t="inlineStr">
+        <is>
+          <t>H6 — How to Use Higgsfield for AI Ad Creatives Without Overcomplicating the Stack</t>
+        </is>
+      </c>
+      <c r="E22" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F22" s="153" t="inlineStr">
+        <is>
+          <t>How-to (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G22" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H22" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="149" t="n"/>
+      <c r="C23" s="150" t="inlineStr">
+        <is>
+          <t>T6, 24/04</t>
+        </is>
+      </c>
+      <c r="D23" s="151" t="inlineStr">
         <is>
           <t>C2 — Dùng AI Tool vận hành cả công ty: Thực tế hay marketing? Review thành thật</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E23" s="152" t="inlineStr">
         <is>
           <t>Cluster C · AI Flywheel</t>
         </is>
       </c>
-      <c r="F17" s="160" t="inlineStr">
+      <c r="F23" s="153" t="inlineStr">
         <is>
           <t>Review (~1,800 từ)</t>
         </is>
       </c>
-      <c r="G17" s="179" t="inlineStr">
+      <c r="G23" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
       </c>
-      <c r="H17" s="162" t="inlineStr">
+      <c r="H23" s="155" t="inlineStr">
         <is>
           <t>📌 Med</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="31.5" customHeight="1" s="115">
-      <c r="B18" s="180" t="n"/>
-      <c r="C18" s="171" t="inlineStr">
-        <is>
-          <t>CN, 19/04</t>
-        </is>
-      </c>
-      <c r="D18" s="172" t="inlineStr">
+    <row r="24" ht="15.75" customHeight="1" s="115">
+      <c r="B24" s="149" t="n"/>
+      <c r="C24" s="150" t="inlineStr">
+        <is>
+          <t>T7, 25/04</t>
+        </is>
+      </c>
+      <c r="D24" s="151" t="inlineStr">
+        <is>
+          <t>H7 — A Creator Workflow Using Higgsfield, Claude, and Automation Tools</t>
+        </is>
+      </c>
+      <c r="E24" s="152" t="inlineStr">
+        <is>
+          <t>Cluster H · Higgsfield</t>
+        </is>
+      </c>
+      <c r="F24" s="153" t="inlineStr">
+        <is>
+          <t>Workflow (~2,200 từ)</t>
+        </is>
+      </c>
+      <c r="G24" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H24" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="149" t="n"/>
+      <c r="C25" s="150" t="inlineStr">
+        <is>
+          <t>CN, 26/04</t>
+        </is>
+      </c>
+      <c r="D25" s="151" t="inlineStr">
         <is>
           <t>B1 — Claude Code là gì? Cách dùng cho người không phải developer — hướng dẫn thực tế</t>
         </is>
       </c>
-      <c r="E18" s="173" t="inlineStr">
+      <c r="E25" s="152" t="inlineStr">
         <is>
           <t>Cluster B · Claude AI</t>
         </is>
       </c>
-      <c r="F18" s="174" t="inlineStr">
+      <c r="F25" s="153" t="inlineStr">
         <is>
           <t>How-to (~2,000 từ)</t>
         </is>
       </c>
-      <c r="G18" s="181" t="inlineStr">
+      <c r="G25" s="154" t="inlineStr">
         <is>
           <t>MoF</t>
         </is>
       </c>
-      <c r="H18" s="176" t="inlineStr">
+      <c r="H25" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="31.5" customHeight="1" s="115">
-      <c r="B19" s="182" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="C19" s="183" t="inlineStr">
-        <is>
-          <t>T2, 20/04</t>
-        </is>
-      </c>
-      <c r="D19" s="184" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="149" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="C26" s="150" t="inlineStr">
+        <is>
+          <t>T2, 27/04</t>
+        </is>
+      </c>
+      <c r="D26" s="151" t="inlineStr">
         <is>
           <t>A4 — Agentic AI có thay thế được nhân viên không? Sự thật phía sau 798K views</t>
         </is>
       </c>
-      <c r="E19" s="185" t="inlineStr">
+      <c r="E26" s="152" t="inlineStr">
         <is>
           <t>Cluster A · Agentic AI</t>
         </is>
       </c>
-      <c r="F19" s="186" t="inlineStr">
+      <c r="F26" s="153" t="inlineStr">
         <is>
           <t>Editorial (~1,500 từ)</t>
         </is>
       </c>
-      <c r="G19" s="187" t="inlineStr">
+      <c r="G26" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H19" s="188" t="inlineStr">
+      <c r="H26" s="155" t="inlineStr">
         <is>
           <t>📌 Med</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="31.5" customHeight="1" s="115">
-      <c r="B20" s="178" t="n"/>
-      <c r="C20" s="157" t="inlineStr">
-        <is>
-          <t>T3, 21/04</t>
-        </is>
-      </c>
-      <c r="D20" s="158" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="149" t="n"/>
+      <c r="C27" s="150" t="inlineStr">
+        <is>
+          <t>T3, 28/04</t>
+        </is>
+      </c>
+      <c r="D27" s="151" t="inlineStr">
         <is>
           <t>C3 — AI Agency 2026: Mô hình kinh doanh mới — chạy agency với 10 AI agents thay nhân sự</t>
         </is>
       </c>
-      <c r="E20" s="159" t="inlineStr">
+      <c r="E27" s="152" t="inlineStr">
         <is>
           <t>Cluster C · AI Flywheel</t>
         </is>
       </c>
-      <c r="F20" s="160" t="inlineStr">
+      <c r="F27" s="153" t="inlineStr">
         <is>
           <t>Case Study (~2,200 từ)</t>
         </is>
       </c>
-      <c r="G20" s="162" t="inlineStr">
+      <c r="G27" s="154" t="inlineStr">
         <is>
           <t>BoF</t>
         </is>
       </c>
-      <c r="H20" s="162" t="inlineStr">
+      <c r="H27" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="31.5" customHeight="1" s="115">
-      <c r="B21" s="180" t="n"/>
-      <c r="C21" s="171" t="inlineStr">
-        <is>
-          <t>T4, 22/04</t>
-        </is>
-      </c>
-      <c r="D21" s="172" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="149" t="n"/>
+      <c r="C28" s="150" t="inlineStr">
+        <is>
+          <t>T4, 29/04</t>
+        </is>
+      </c>
+      <c r="D28" s="151" t="inlineStr">
         <is>
           <t>B4 — Claude API: Hướng dẫn tích hợp vào workflow của bạn (không cần biết code)</t>
         </is>
       </c>
-      <c r="E21" s="173" t="inlineStr">
+      <c r="E28" s="152" t="inlineStr">
         <is>
           <t>Cluster B · Claude AI</t>
         </is>
       </c>
-      <c r="F21" s="174" t="inlineStr">
+      <c r="F28" s="153" t="inlineStr">
         <is>
           <t>Tutorial (~2,000 từ)</t>
         </is>
       </c>
-      <c r="G21" s="189" t="inlineStr">
+      <c r="G28" s="154" t="inlineStr">
         <is>
           <t>BoF</t>
         </is>
       </c>
-      <c r="H21" s="176" t="inlineStr">
+      <c r="H28" s="155" t="inlineStr">
         <is>
           <t>⚡ High</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="31.5" customHeight="1" s="115">
-      <c r="B22" s="190" t="n"/>
-      <c r="C22" s="191" t="inlineStr">
-        <is>
-          <t>T5, 23/04</t>
-        </is>
-      </c>
-      <c r="D22" s="192" t="inlineStr">
-        <is>
-          <t>D-Flex — Bài tin tức linh hoạt theo sự kiện AI tuần đó (chủ đề xác định T4/05/05)</t>
-        </is>
-      </c>
-      <c r="E22" s="193" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="149" t="n"/>
+      <c r="C29" s="150" t="inlineStr">
+        <is>
+          <t>T5, 30/04</t>
+        </is>
+      </c>
+      <c r="D29" s="151" t="inlineStr">
+        <is>
+          <t>D-Flex — Bài tin tức linh hoạt theo sự kiện AI tuần đó (chủ đề xác định theo news cycle)</t>
+        </is>
+      </c>
+      <c r="E29" s="152" t="inlineStr">
         <is>
           <t>Cluster D · News</t>
         </is>
       </c>
-      <c r="F22" s="194" t="inlineStr">
+      <c r="F29" s="153" t="inlineStr">
         <is>
           <t>News Flex (~1,000 từ)</t>
         </is>
       </c>
-      <c r="G22" s="195" t="inlineStr">
+      <c r="G29" s="154" t="inlineStr">
         <is>
           <t>ToF</t>
         </is>
       </c>
-      <c r="H22" s="196" t="inlineStr">
+      <c r="H29" s="155" t="inlineStr">
         <is>
           <t>📰 Flex</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="115">
-      <c r="B24" s="197" t="inlineStr">
-        <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. Từ 10/04 chuyển sang nhịp 1 bài/ngày. Các bài đã viết nhưng chưa đăng phải đối chiếu thêm với repo trước khi publish.</t>
-        </is>
-      </c>
-    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1 và H1 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B24:H24"/>
     <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2383,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:K21"/>
+  <dimension ref="A2:K59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -2402,7 +2637,7 @@
     <row r="2" ht="39.75" customHeight="1" s="115">
       <c r="B2" s="147" t="inlineStr">
         <is>
-          <t>DANH SÁCH 20 BÀI VIẾT — CHI TIẾT TRIỂN KHAI</t>
+          <t>DANH SÁCH 27 BÀI VIẾT — CHI TIẾT TRIỂN KHAI</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2844,7 @@
       </c>
       <c r="I7" s="153" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="J7" s="201" t="inlineStr">
@@ -2664,7 +2899,7 @@
       </c>
       <c r="I8" s="153" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="J8" s="201" t="inlineStr">
@@ -2719,7 +2954,7 @@
       </c>
       <c r="I9" s="153" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="J9" s="201" t="inlineStr">
@@ -2829,7 +3064,7 @@
       </c>
       <c r="I11" s="174" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="J11" s="205" t="inlineStr">
@@ -2884,7 +3119,7 @@
       </c>
       <c r="I12" s="174" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="J12" s="205" t="inlineStr">
@@ -2939,7 +3174,7 @@
       </c>
       <c r="I13" s="174" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="J13" s="205" t="inlineStr">
@@ -2994,7 +3229,7 @@
       </c>
       <c r="I14" s="174" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="J14" s="205" t="inlineStr">
@@ -3159,7 +3394,7 @@
       </c>
       <c r="I17" s="160" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="J17" s="209" t="inlineStr">
@@ -3214,7 +3449,7 @@
       </c>
       <c r="I18" s="160" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="J18" s="209" t="inlineStr">
@@ -3324,7 +3559,7 @@
       </c>
       <c r="I20" s="194" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="J20" s="213" t="inlineStr">
@@ -3394,6 +3629,422 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="B22" s="211" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C22" s="212" t="inlineStr">
+        <is>
+          <t>What Is Higgsfield AI? A Practical Guide for Creators</t>
+        </is>
+      </c>
+      <c r="D22" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E22" s="194" t="inlineStr">
+        <is>
+          <t>Guide · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F22" s="194" t="inlineStr">
+        <is>
+          <t>what is higgsfield ai</t>
+        </is>
+      </c>
+      <c r="G22" s="213" t="inlineStr">
+        <is>
+          <t>→ H2 (beginner follow-up), affiliate-workflow-for-content-creators (cross-cluster)
+← H4/H5 link back to H1</t>
+        </is>
+      </c>
+      <c r="H22" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+View Higgsfield tool page</t>
+        </is>
+      </c>
+      <c r="I22" s="194" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="J22" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: understand the tool and where it fits</t>
+        </is>
+      </c>
+      <c r="K22" s="214" t="inlineStr">
+        <is>
+          <t>🟡 Đã viết / chờ đăng</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="211" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="C23" s="212" t="inlineStr">
+        <is>
+          <t>Higgsfield for Beginners: What to Test First</t>
+        </is>
+      </c>
+      <c r="D23" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E23" s="194" t="inlineStr">
+        <is>
+          <t>Guide · 1,600 từ</t>
+        </is>
+      </c>
+      <c r="F23" s="194" t="inlineStr">
+        <is>
+          <t>higgsfield for beginners</t>
+        </is>
+      </c>
+      <c r="G23" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), tools/higgsfield (supporting path)
+← H1 links forward to H2</t>
+        </is>
+      </c>
+      <c r="H23" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF/MoF)
+Start with the tool page</t>
+        </is>
+      </c>
+      <c r="I23" s="194" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="J23" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: reduce beginner friction</t>
+        </is>
+      </c>
+      <c r="K23" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="211" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="C24" s="212" t="inlineStr">
+        <is>
+          <t>Best Use Cases for Higgsfield in Short-Form Content Workflows</t>
+        </is>
+      </c>
+      <c r="D24" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E24" s="194" t="inlineStr">
+        <is>
+          <t>Guide · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F24" s="194" t="inlineStr">
+        <is>
+          <t>higgsfield use cases</t>
+        </is>
+      </c>
+      <c r="G24" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), affiliate-workflow-for-content-creators (cross-cluster)
+← H2 links forward to H3</t>
+        </is>
+      </c>
+      <c r="H24" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See workflow fit</t>
+        </is>
+      </c>
+      <c r="I24" s="194" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="J24" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: evaluate practical use cases</t>
+        </is>
+      </c>
+      <c r="K24" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="211" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C25" s="212" t="inlineStr">
+        <is>
+          <t>Higgsfield vs Runway: Which One Fits Faster Creator Workflows?</t>
+        </is>
+      </c>
+      <c r="D25" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E25" s="194" t="inlineStr">
+        <is>
+          <t>Comparison · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F25" s="194" t="inlineStr">
+        <is>
+          <t>higgsfield vs runway</t>
+        </is>
+      </c>
+      <c r="G25" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), H5 (alternatives)
+← H1 links forward to H4</t>
+        </is>
+      </c>
+      <c r="H25" s="213" t="inlineStr">
+        <is>
+          <t>Comparison CTA (MoF)
+Choose the better fit</t>
+        </is>
+      </c>
+      <c r="I25" s="194" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="J25" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: compare before choosing</t>
+        </is>
+      </c>
+      <c r="K25" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="211" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="C26" s="212" t="inlineStr">
+        <is>
+          <t>Higgsfield Alternatives: When to Choose Another AI Visual Tool</t>
+        </is>
+      </c>
+      <c r="D26" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E26" s="194" t="inlineStr">
+        <is>
+          <t>Comparison · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F26" s="194" t="inlineStr">
+        <is>
+          <t>higgsfield alternatives</t>
+        </is>
+      </c>
+      <c r="G26" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), H4 (comparison)
+← H4 links to H5</t>
+        </is>
+      </c>
+      <c r="H26" s="213" t="inlineStr">
+        <is>
+          <t>Comparison CTA (MoF)
+Review alternative paths</t>
+        </is>
+      </c>
+      <c r="I26" s="194" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="J26" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: evaluate alternatives</t>
+        </is>
+      </c>
+      <c r="K26" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="211" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="C27" s="212" t="inlineStr">
+        <is>
+          <t>How to Use Higgsfield for AI Ad Creatives Without Overcomplicating the Stack</t>
+        </is>
+      </c>
+      <c r="D27" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E27" s="194" t="inlineStr">
+        <is>
+          <t>How-to · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F27" s="194" t="inlineStr">
+        <is>
+          <t>how to use higgsfield</t>
+        </is>
+      </c>
+      <c r="G27" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), C2 (cross-cluster)
+← H3 links forward to H6</t>
+        </is>
+      </c>
+      <c r="H27" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF/BoF)
+Apply it in a real stack</t>
+        </is>
+      </c>
+      <c r="I27" s="194" t="inlineStr">
+        <is>
+          <t>23/04/2026</t>
+        </is>
+      </c>
+      <c r="J27" s="213" t="inlineStr">
+        <is>
+          <t>Instructional · MoF-BoF
+Intent: apply the tool in marketing workflows</t>
+        </is>
+      </c>
+      <c r="K27" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="211" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="C28" s="212" t="inlineStr">
+        <is>
+          <t>A Creator Workflow Using Higgsfield, Claude, and Automation Tools</t>
+        </is>
+      </c>
+      <c r="D28" s="193" t="inlineStr">
+        <is>
+          <t>Cluster H</t>
+        </is>
+      </c>
+      <c r="E28" s="194" t="inlineStr">
+        <is>
+          <t>Workflow · 2,200 từ</t>
+        </is>
+      </c>
+      <c r="F28" s="194" t="inlineStr">
+        <is>
+          <t>higgsfield workflow</t>
+        </is>
+      </c>
+      <c r="G28" s="213" t="inlineStr">
+        <is>
+          <t>→ H1 (pillar), B0 (cross-cluster)
+← H6 links forward to H7</t>
+        </is>
+      </c>
+      <c r="H28" s="213" t="inlineStr">
+        <is>
+          <t>Workflow CTA (MoF)
+Go from tool to system</t>
+        </is>
+      </c>
+      <c r="I28" s="194" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="J28" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: fit Higgsfield into a broader stack</t>
+        </is>
+      </c>
+      <c r="K28" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:K2"/>

</xml_diff>

<commit_message>
Add scheduled Higgsfield beginner guide
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -1691,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:H34"/>
+  <dimension ref="B2:H31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -2590,17 +2590,13 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1 và H1 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
+      <c r="B31" s="114" t="inlineStr">
+        <is>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1 và H2 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:H2"/>
@@ -2618,7 +2614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:K59"/>
+  <dimension ref="B2:K28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -3735,7 +3731,7 @@
       </c>
       <c r="K23" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>
@@ -4014,37 +4010,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:K2"/>

</xml_diff>

<commit_message>
Add scheduled Higgsfield use cases post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1 và H2 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2 và H3 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="K24" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Higgsfield comparison post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2 và H3 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3 và H4 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="K25" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Higgsfield alternatives post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3 và H4 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4 và H5 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="K26" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Higgsfield ad creative guide
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4 và H5 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4, H5 và H6 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="K27" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Higgsfield workflow post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4, H5 và H6 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="K28" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Agentic AI monetization post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2593,7 +2593,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="K16" s="210" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Claude comparison post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -1345,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:G26"/>
+  <dimension ref="B2:G28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -1659,6 +1659,13 @@
       <c r="B26" s="146" t="inlineStr">
         <is>
           <t>Dữ liệu nguồn: plan_content_moltyflywheel.html · shared_context.json · 30 video YouTube phân tích (Agentic AI + Claude AI · ~10M+ views)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="114" t="inlineStr">
+        <is>
+          <t>[10/04/2026 00:10] | A1 | 5 ứng dụng Agentic AI trong doanh nghiệp... | ✅ Đã đăng (10/04)</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2803,7 @@
       </c>
       <c r="K6" s="202" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (10/04)</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3133,7 @@
       </c>
       <c r="K12" s="206" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled AI agent vs assistant post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="K7" s="202" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled AI agent tutorial post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="K8" s="202" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Claude prompts post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="K13" s="206" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Qwen3 analysis post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="K20" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled AI operations review post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="K17" s="210" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Claude Code guide
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="K11" s="206" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Agentic AI workforce post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="K9" s="202" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled AI agency post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2600,7 +2600,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="K18" s="210" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add scheduled Claude API workflow post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -1345,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:G28"/>
+  <dimension ref="B2:G30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -1666,6 +1666,20 @@
       <c r="B28" s="114" t="inlineStr">
         <is>
           <t>[10/04/2026 00:10] | A1 | 5 ứng dụng Agentic AI trong doanh nghiệp... | ✅ Đã đăng (10/04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="114" t="inlineStr">
+        <is>
+          <t>[10/04/2026 01:11] | A1 | 5 ứng dụng Agentic AI trong doanh nghiệp... | ✅ Đã đăng (10/04) (confirmed — đã đăng từ lần chạy trước)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="114" t="inlineStr">
+        <is>
+          <t>[10/04/2026 01:21] | A1 | 5 ứng dụng Agentic AI trong doanh nghiệp... | ✅ Đã đăng (10/04) (confirmed — đã đăng từ lần chạy trước)</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2614,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày.</t>
+          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:K28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -3243,7 +3257,7 @@
       </c>
       <c r="K14" s="206" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>🟡 Đã viết / chờ đăng</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish April 11 Claude roundup
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2614,7 +2614,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3 và B0 đã live. A1, D1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
+          <t>Ghi chú: A0, C0, D3, B0 và D1 đã live. A1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="K19" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (11/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish April 12 Agentic AI post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2614,7 +2614,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3, B0 và D1 đã live. A1, C1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
+          <t>Ghi chú: A0, C0, D3, B0, D1 và C1 đã live. A1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="K16" s="210" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (12/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish April 13 Higgsfield guide
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2614,7 +2614,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3, B0, D1 và C1 đã live. A1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H1, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
+          <t>Ghi chú: A0, C0, D3, B0, D1, C1 và H1 đã live. A1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
         </is>
       </c>
     </row>
@@ -3697,7 +3697,7 @@
       </c>
       <c r="K22" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (13/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish overdue April blog posts
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2614,7 +2614,7 @@
     <row r="31">
       <c r="B31" s="114" t="inlineStr">
         <is>
-          <t>Ghi chú: A0, C0, D3, B0, D1, C1 và H1 đã live. A1, B2, A2, A3, B3, D2, C2, B1, A4, C3, B4, H2, H3, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
+          <t>Ghi chú: A0, C0, D3, B0, D1, C1, H1, B2, H2, A2 và H3 đã live. A1, A3, B3, D2, C2, B1, A4, C3, B4, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="K7" s="202" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (17/04)</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="K12" s="206" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (17/04)</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="K23" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (17/04)</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="K24" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (17/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish overdue posts through April 24
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -2635,7 +2635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="B2:K28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="K8" s="202" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="K13" s="206" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="K17" s="210" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="K20" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="K25" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="K26" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="K27" s="214" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (24/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Port May 2026 plan into workbook
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -19,7 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="29">
     <font>
       <name val="Calibri"/>
@@ -326,7 +328,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -397,6 +399,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -408,7 +434,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1091,6 +1117,12 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1712,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:H31"/>
+  <dimension ref="B2:H62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -1728,7 +1760,7 @@
     <row r="2" ht="39.75" customHeight="1" s="115">
       <c r="B2" s="147" t="inlineStr">
         <is>
-          <t>LỊCH XUẤT BẢN — DAILY CADENCE (April 6 – April 30, 2026)</t>
+          <t>LỊCH XUẤT BẢN — DAILY CADENCE (April 6 – May 31, 2026)</t>
         </is>
       </c>
     </row>
@@ -2612,16 +2644,1059 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="114" t="inlineStr">
-        <is>
-          <t>Ghi chú: A0, C0, D3, B0, D1, C1, H1, B2, H2, A2 và H3 đã live. A1, A3, B3, D2, C2, B1, A4, C3, B4, H4, H5, H6 và H7 đã viết nhưng chưa đăng. Từ 13/04, series Higgsfield được xen kẽ với queue hiện có ở nhịp 1 bài/ngày. Queue hiện tại đã viết kín lịch đến 29/04.</t>
+      <c r="B31" s="149" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>T6, 01/05</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>A5 — What Is Abacus AI? A Practical Guide to Models, Agents, and the Managed Claw Path</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Guide (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>🔥 Hot</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="149" t="n"/>
+      <c r="C32" s="150" t="inlineStr">
+        <is>
+          <t>T7, 02/05</t>
+        </is>
+      </c>
+      <c r="D32" s="151" t="inlineStr">
+        <is>
+          <t>T1 — What Is Topview AI? A Practical Guide for Product Videos and UGC Ad Creatives</t>
+        </is>
+      </c>
+      <c r="E32" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F32" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G32" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H32" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="149" t="n"/>
+      <c r="C33" s="150" t="inlineStr">
+        <is>
+          <t>CN, 03/05</t>
+        </is>
+      </c>
+      <c r="D33" s="151" t="inlineStr">
+        <is>
+          <t>O1 — How to Choose Between Programs, Offers, and Tools Without Wasting Time</t>
+        </is>
+      </c>
+      <c r="E33" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F33" s="153" t="inlineStr">
+        <is>
+          <t>Framework (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G33" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H33" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="149" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="C34" s="150" t="inlineStr">
+        <is>
+          <t>T2, 04/05</t>
+        </is>
+      </c>
+      <c r="D34" s="151" t="inlineStr">
+        <is>
+          <t>P1 — Best AI Tools for Affiliate Content Workflows in 2026</t>
+        </is>
+      </c>
+      <c r="E34" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F34" s="153" t="inlineStr">
+        <is>
+          <t>Commercial Guide (~2,200 từ)</t>
+        </is>
+      </c>
+      <c r="G34" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H34" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="149" t="n"/>
+      <c r="C35" s="150" t="inlineStr">
+        <is>
+          <t>T3, 05/05</t>
+        </is>
+      </c>
+      <c r="D35" s="151" t="inlineStr">
+        <is>
+          <t>A6 — Abacus AI vs OpenClaw: When a Managed Agent Platform Makes More Sense</t>
+        </is>
+      </c>
+      <c r="E35" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F35" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G35" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H35" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="149" t="n"/>
+      <c r="C36" s="150" t="inlineStr">
+        <is>
+          <t>T4, 06/05</t>
+        </is>
+      </c>
+      <c r="D36" s="151" t="inlineStr">
+        <is>
+          <t>T2 — Topview AI for Beginners: What to Test First Before You Commit to a Workflow</t>
+        </is>
+      </c>
+      <c r="E36" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F36" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~1,700 từ)</t>
+        </is>
+      </c>
+      <c r="G36" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H36" s="155" t="inlineStr">
+        <is>
+          <t>✨ New</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="149" t="n"/>
+      <c r="C37" s="150" t="inlineStr">
+        <is>
+          <t>T5, 07/05</t>
+        </is>
+      </c>
+      <c r="D37" s="151" t="inlineStr">
+        <is>
+          <t>N1 — Weekly AI Systems Roundup: Models, Agents, and Tool Moves Worth Tracking</t>
+        </is>
+      </c>
+      <c r="E37" s="152" t="inlineStr">
+        <is>
+          <t>Track N · News</t>
+        </is>
+      </c>
+      <c r="F37" s="153" t="inlineStr">
+        <is>
+          <t>Roundup (~1,200 từ)</t>
+        </is>
+      </c>
+      <c r="G37" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H37" s="155" t="inlineStr">
+        <is>
+          <t>📰 News</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="149" t="n"/>
+      <c r="C38" s="150" t="inlineStr">
+        <is>
+          <t>T6, 08/05</t>
+        </is>
+      </c>
+      <c r="D38" s="151" t="inlineStr">
+        <is>
+          <t>O2 — Best Offer Page Type for Your Current Stage: Beginner Fit, Comparison, or Niche Path?</t>
+        </is>
+      </c>
+      <c r="E38" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F38" s="153" t="inlineStr">
+        <is>
+          <t>Decision Support (~1,900 từ)</t>
+        </is>
+      </c>
+      <c r="G38" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H38" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="149" t="n"/>
+      <c r="C39" s="150" t="inlineStr">
+        <is>
+          <t>T7, 09/05</t>
+        </is>
+      </c>
+      <c r="D39" s="151" t="inlineStr">
+        <is>
+          <t>P2 — ConvertKit vs Beehiiv for AI Content Operators: Which One Fits Better?</t>
+        </is>
+      </c>
+      <c r="E39" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F39" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G39" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H39" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="149" t="n"/>
+      <c r="C40" s="150" t="inlineStr">
+        <is>
+          <t>CN, 10/05</t>
+        </is>
+      </c>
+      <c r="D40" s="151" t="inlineStr">
+        <is>
+          <t>A7 — Best Use Cases for Abacus AI in Small Operator Teams</t>
+        </is>
+      </c>
+      <c r="E40" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F40" s="153" t="inlineStr">
+        <is>
+          <t>Use Case Guide (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G40" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H40" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="149" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C41" s="150" t="inlineStr">
+        <is>
+          <t>T2, 11/05</t>
+        </is>
+      </c>
+      <c r="D41" s="151" t="inlineStr">
+        <is>
+          <t>T3 — Best Use Cases for Topview AI in Affiliate and Ecommerce Creative Workflows</t>
+        </is>
+      </c>
+      <c r="E41" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F41" s="153" t="inlineStr">
+        <is>
+          <t>Use Case Guide (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G41" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H41" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="149" t="n"/>
+      <c r="C42" s="150" t="inlineStr">
+        <is>
+          <t>T3, 12/05</t>
+        </is>
+      </c>
+      <c r="D42" s="151" t="inlineStr">
+        <is>
+          <t>O3 — Affiliate Program vs Affiliate Platform: What You Actually Need to Decide First</t>
+        </is>
+      </c>
+      <c r="E42" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F42" s="153" t="inlineStr">
+        <is>
+          <t>Explainer (~1,900 từ)</t>
+        </is>
+      </c>
+      <c r="G42" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H42" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="149" t="n"/>
+      <c r="C43" s="150" t="inlineStr">
+        <is>
+          <t>T4, 13/05</t>
+        </is>
+      </c>
+      <c r="D43" s="151" t="inlineStr">
+        <is>
+          <t>P3 — n8n vs Make for Lean AI Operations: Which Automation Layer Fits Better?</t>
+        </is>
+      </c>
+      <c r="E43" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F43" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G43" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H43" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="149" t="n"/>
+      <c r="C44" s="150" t="inlineStr">
+        <is>
+          <t>T5, 14/05</t>
+        </is>
+      </c>
+      <c r="D44" s="151" t="inlineStr">
+        <is>
+          <t>N2 — Weekly AI Tool Signal Check: What Changed and What Actually Matters</t>
+        </is>
+      </c>
+      <c r="E44" s="152" t="inlineStr">
+        <is>
+          <t>Track N · News</t>
+        </is>
+      </c>
+      <c r="F44" s="153" t="inlineStr">
+        <is>
+          <t>Roundup (~1,200 từ)</t>
+        </is>
+      </c>
+      <c r="G44" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H44" s="155" t="inlineStr">
+        <is>
+          <t>📰 News</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="149" t="n"/>
+      <c r="C45" s="150" t="inlineStr">
+        <is>
+          <t>T6, 15/05</t>
+        </is>
+      </c>
+      <c r="D45" s="151" t="inlineStr">
+        <is>
+          <t>A8 — Abacus AI Model Stack Explained: When Multi-Model Access Is Actually Useful</t>
+        </is>
+      </c>
+      <c r="E45" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F45" s="153" t="inlineStr">
+        <is>
+          <t>Explainer (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G45" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H45" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="149" t="n"/>
+      <c r="C46" s="150" t="inlineStr">
+        <is>
+          <t>T7, 16/05</t>
+        </is>
+      </c>
+      <c r="D46" s="151" t="inlineStr">
+        <is>
+          <t>T4 — Topview AI vs Higgsfield: Which Tool Fits Marketing Video Workflows Better?</t>
+        </is>
+      </c>
+      <c r="E46" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F46" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G46" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H46" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="149" t="n"/>
+      <c r="C47" s="150" t="inlineStr">
+        <is>
+          <t>CN, 17/05</t>
+        </is>
+      </c>
+      <c r="D47" s="151" t="inlineStr">
+        <is>
+          <t>O4 — Best Affiliate Programs by Workflow Type, Not Just by Commission Size</t>
+        </is>
+      </c>
+      <c r="E47" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F47" s="153" t="inlineStr">
+        <is>
+          <t>Commercial Guide (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G47" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H47" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="149" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="C48" s="150" t="inlineStr">
+        <is>
+          <t>T2, 18/05</t>
+        </is>
+      </c>
+      <c r="D48" s="151" t="inlineStr">
+        <is>
+          <t>P4 — Best AI Writing Tool for Program Reviews and Comparison Posts in 2026</t>
+        </is>
+      </c>
+      <c r="E48" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F48" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G48" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H48" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="149" t="n"/>
+      <c r="C49" s="150" t="inlineStr">
+        <is>
+          <t>T3, 19/05</t>
+        </is>
+      </c>
+      <c r="D49" s="151" t="inlineStr">
+        <is>
+          <t>A9 — How to Evaluate a Hosted Agent Platform Before Replacing Your Current Stack</t>
+        </is>
+      </c>
+      <c r="E49" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F49" s="153" t="inlineStr">
+        <is>
+          <t>Framework (~1,900 từ)</t>
+        </is>
+      </c>
+      <c r="G49" s="154" t="inlineStr">
+        <is>
+          <t>BoF</t>
+        </is>
+      </c>
+      <c r="H49" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="149" t="n"/>
+      <c r="C50" s="150" t="inlineStr">
+        <is>
+          <t>T4, 20/05</t>
+        </is>
+      </c>
+      <c r="D50" s="151" t="inlineStr">
+        <is>
+          <t>T5 — Topview AI Alternatives: When Another Visual Tool Is the Better Choice</t>
+        </is>
+      </c>
+      <c r="E50" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F50" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~1,800 từ)</t>
+        </is>
+      </c>
+      <c r="G50" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H50" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="149" t="n"/>
+      <c r="C51" s="150" t="inlineStr">
+        <is>
+          <t>T5, 21/05</t>
+        </is>
+      </c>
+      <c r="D51" s="151" t="inlineStr">
+        <is>
+          <t>N3 — Weekly AI Market Analysis: Which Product Signals Are Real and Which Are Just Launch Noise?</t>
+        </is>
+      </c>
+      <c r="E51" s="152" t="inlineStr">
+        <is>
+          <t>Track N · News</t>
+        </is>
+      </c>
+      <c r="F51" s="153" t="inlineStr">
+        <is>
+          <t>Analysis (~1,400 từ)</t>
+        </is>
+      </c>
+      <c r="G51" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H51" s="155" t="inlineStr">
+        <is>
+          <t>📰 News</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="149" t="n"/>
+      <c r="C52" s="150" t="inlineStr">
+        <is>
+          <t>T6, 22/05</t>
+        </is>
+      </c>
+      <c r="D52" s="151" t="inlineStr">
+        <is>
+          <t>O5 — Recurring vs High-Ticket Offers in 2026: Which Route Fits Your Current System?</t>
+        </is>
+      </c>
+      <c r="E52" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F52" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G52" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H52" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="149" t="n"/>
+      <c r="C53" s="150" t="inlineStr">
+        <is>
+          <t>T7, 23/05</t>
+        </is>
+      </c>
+      <c r="D53" s="151" t="inlineStr">
+        <is>
+          <t>P5 — Claude Pro vs ChatLLM Teams: Which Operator Layer Fits Better for Daily Work?</t>
+        </is>
+      </c>
+      <c r="E53" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F53" s="153" t="inlineStr">
+        <is>
+          <t>Comparison (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G53" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H53" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="149" t="n"/>
+      <c r="C54" s="150" t="inlineStr">
+        <is>
+          <t>CN, 24/05</t>
+        </is>
+      </c>
+      <c r="D54" s="151" t="inlineStr">
+        <is>
+          <t>A10 — A Practical Abacus AI Workflow for Research, Writing, and Agent-Assisted Ops</t>
+        </is>
+      </c>
+      <c r="E54" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F54" s="153" t="inlineStr">
+        <is>
+          <t>Workflow (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G54" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H54" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="149" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="C55" s="150" t="inlineStr">
+        <is>
+          <t>T2, 25/05</t>
+        </is>
+      </c>
+      <c r="D55" s="151" t="inlineStr">
+        <is>
+          <t>T6 — How to Use Topview AI for Affiliate Product Videos Without Overbuilding the Stack</t>
+        </is>
+      </c>
+      <c r="E55" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F55" s="153" t="inlineStr">
+        <is>
+          <t>How-to (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G55" s="154" t="inlineStr">
+        <is>
+          <t>MoF/BoF</t>
+        </is>
+      </c>
+      <c r="H55" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="149" t="n"/>
+      <c r="C56" s="150" t="inlineStr">
+        <is>
+          <t>T3, 26/05</t>
+        </is>
+      </c>
+      <c r="D56" s="151" t="inlineStr">
+        <is>
+          <t>O6 — The Fastest Way to Find Your Best Affiliate Fit Without Starting Over Repeatedly</t>
+        </is>
+      </c>
+      <c r="E56" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F56" s="153" t="inlineStr">
+        <is>
+          <t>Decision Support (~1,900 từ)</t>
+        </is>
+      </c>
+      <c r="G56" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H56" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="149" t="n"/>
+      <c r="C57" s="150" t="inlineStr">
+        <is>
+          <t>T4, 27/05</t>
+        </is>
+      </c>
+      <c r="D57" s="151" t="inlineStr">
+        <is>
+          <t>P6 — Best AI Tools for Landing Pages, Funnels, and Conversion Assets in 2026</t>
+        </is>
+      </c>
+      <c r="E57" s="152" t="inlineStr">
+        <is>
+          <t>Track P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="F57" s="153" t="inlineStr">
+        <is>
+          <t>Commercial Guide (~2,100 từ)</t>
+        </is>
+      </c>
+      <c r="G57" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H57" s="155" t="inlineStr">
+        <is>
+          <t>⚡ High</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="149" t="n"/>
+      <c r="C58" s="150" t="inlineStr">
+        <is>
+          <t>T5, 28/05</t>
+        </is>
+      </c>
+      <c r="D58" s="151" t="inlineStr">
+        <is>
+          <t>N4 — Weekly AI Systems Roundup: Agent Products, Creator Tools, and Search Shifts</t>
+        </is>
+      </c>
+      <c r="E58" s="152" t="inlineStr">
+        <is>
+          <t>Track N · News</t>
+        </is>
+      </c>
+      <c r="F58" s="153" t="inlineStr">
+        <is>
+          <t>Roundup (~1,200 từ)</t>
+        </is>
+      </c>
+      <c r="G58" s="154" t="inlineStr">
+        <is>
+          <t>ToF</t>
+        </is>
+      </c>
+      <c r="H58" s="155" t="inlineStr">
+        <is>
+          <t>📰 News</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="149" t="n"/>
+      <c r="C59" s="150" t="inlineStr">
+        <is>
+          <t>T6, 29/05</t>
+        </is>
+      </c>
+      <c r="D59" s="151" t="inlineStr">
+        <is>
+          <t>A11 — Abacus AI for Non-Developers: Where It Helps and Where It Is Overkill</t>
+        </is>
+      </c>
+      <c r="E59" s="152" t="inlineStr">
+        <is>
+          <t>Track A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="F59" s="153" t="inlineStr">
+        <is>
+          <t>Guide (~1,900 từ)</t>
+        </is>
+      </c>
+      <c r="G59" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H59" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="149" t="n"/>
+      <c r="C60" s="150" t="inlineStr">
+        <is>
+          <t>T7, 30/05</t>
+        </is>
+      </c>
+      <c r="D60" s="151" t="inlineStr">
+        <is>
+          <t>T7 — A Creator Workflow Using Topview AI, Claude, and Automation Tools</t>
+        </is>
+      </c>
+      <c r="E60" s="152" t="inlineStr">
+        <is>
+          <t>Track T · Topview AI</t>
+        </is>
+      </c>
+      <c r="F60" s="153" t="inlineStr">
+        <is>
+          <t>Workflow (~2,200 từ)</t>
+        </is>
+      </c>
+      <c r="G60" s="154" t="inlineStr">
+        <is>
+          <t>MoF</t>
+        </is>
+      </c>
+      <c r="H60" s="155" t="inlineStr">
+        <is>
+          <t>📌 Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="149" t="n"/>
+      <c r="C61" s="150" t="inlineStr">
+        <is>
+          <t>CN, 31/05</t>
+        </is>
+      </c>
+      <c r="D61" s="151" t="inlineStr">
+        <is>
+          <t>O7 — Programs, Tools, and Offers: How the MoltyFlywheel System Fits Together in Practice</t>
+        </is>
+      </c>
+      <c r="E61" s="152" t="inlineStr">
+        <is>
+          <t>Track O · Decision Support</t>
+        </is>
+      </c>
+      <c r="F61" s="153" t="inlineStr">
+        <is>
+          <t>System Guide (~2,000 từ)</t>
+        </is>
+      </c>
+      <c r="G61" s="154" t="inlineStr">
+        <is>
+          <t>ToF/MoF</t>
+        </is>
+      </c>
+      <c r="H61" s="155" t="inlineStr">
+        <is>
+          <t>🏷 Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="149" t="inlineStr">
+        <is>
+          <t>Ghi chú: Queue tháng 4 đã được port và tháng 5 đã được lên kế hoạch daily cadence 1 bài/ngày. Các bài tháng 5 hiện ở trạng thái planned và chưa viết trừ khi có task sản xuất riêng.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="B62:H62"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2635,7 +3710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:K28"/>
+  <dimension ref="B2:K59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -4028,6 +5103,1649 @@
       <c r="K28" s="214" t="inlineStr">
         <is>
           <t>✅ Đã đăng (25/04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="211" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C29" s="212" t="inlineStr">
+        <is>
+          <t>What Is Abacus AI? A Practical Guide to Models, Agents, and the Managed Claw Path</t>
+        </is>
+      </c>
+      <c r="D29" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E29" s="194" t="inlineStr">
+        <is>
+          <t>Guide  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F29" s="194" t="inlineStr">
+        <is>
+          <t>what is abacus ai</t>
+        </is>
+      </c>
+      <c r="G29" s="213" t="inlineStr">
+        <is>
+          <t>→ A6, A8, /tools/abacus-ai/
+← May Track A links back to A5</t>
+        </is>
+      </c>
+      <c r="H29" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+View Abacus AI tool page</t>
+        </is>
+      </c>
+      <c r="I29" s="230" t="n">
+        <v>46143</v>
+      </c>
+      <c r="J29" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: understand Abacus AI and managed agent fit</t>
+        </is>
+      </c>
+      <c r="K29" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="211" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C30" s="212" t="inlineStr">
+        <is>
+          <t>What Is Topview AI? A Practical Guide for Product Videos and UGC Ad Creatives</t>
+        </is>
+      </c>
+      <c r="D30" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E30" s="194" t="inlineStr">
+        <is>
+          <t>Guide  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F30" s="194" t="inlineStr">
+        <is>
+          <t>what is topview ai</t>
+        </is>
+      </c>
+      <c r="G30" s="213" t="inlineStr">
+        <is>
+          <t>→ T2, T4, /tools/topview-ai/
+← May Track T links back to T1</t>
+        </is>
+      </c>
+      <c r="H30" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+View Topview AI tool page</t>
+        </is>
+      </c>
+      <c r="I30" s="230" t="n">
+        <v>46144</v>
+      </c>
+      <c r="J30" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: understand Topview AI and creator fit</t>
+        </is>
+      </c>
+      <c r="K30" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="211" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C31" s="212" t="inlineStr">
+        <is>
+          <t>How to Choose Between Programs, Offers, and Tools Without Wasting Time</t>
+        </is>
+      </c>
+      <c r="D31" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E31" s="194" t="inlineStr">
+        <is>
+          <t>Framework  · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F31" s="194" t="inlineStr">
+        <is>
+          <t>programs vs offers vs tools</t>
+        </is>
+      </c>
+      <c r="G31" s="213" t="inlineStr">
+        <is>
+          <t>→ O2, O7, /tools/, /offers/
+← decision-support posts link back to O1</t>
+        </is>
+      </c>
+      <c r="H31" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Choose the right route</t>
+        </is>
+      </c>
+      <c r="I31" s="230" t="n">
+        <v>46145</v>
+      </c>
+      <c r="J31" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: reduce route confusion</t>
+        </is>
+      </c>
+      <c r="K31" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="211" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C32" s="212" t="inlineStr">
+        <is>
+          <t>Best AI Tools for Affiliate Content Workflows in 2026</t>
+        </is>
+      </c>
+      <c r="D32" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E32" s="194" t="inlineStr">
+        <is>
+          <t>Commercial Guide  · 2,200 từ</t>
+        </is>
+      </c>
+      <c r="F32" s="194" t="inlineStr">
+        <is>
+          <t>best ai tools for affiliate content</t>
+        </is>
+      </c>
+      <c r="G32" s="213" t="inlineStr">
+        <is>
+          <t>→ P2, P6, /offers/affiliate-tools-for-content-creators/
+← workflow posts link back to P1</t>
+        </is>
+      </c>
+      <c r="H32" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See creator tools offer page</t>
+        </is>
+      </c>
+      <c r="I32" s="230" t="n">
+        <v>46146</v>
+      </c>
+      <c r="J32" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: choose tools for affiliate workflow</t>
+        </is>
+      </c>
+      <c r="K32" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="211" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="C33" s="212" t="inlineStr">
+        <is>
+          <t>Abacus AI vs OpenClaw: When a Managed Agent Platform Makes More Sense</t>
+        </is>
+      </c>
+      <c r="D33" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E33" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F33" s="194" t="inlineStr">
+        <is>
+          <t>abacus ai vs openclaw</t>
+        </is>
+      </c>
+      <c r="G33" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, A9, how-openclaw-generates-1-blog-post-per-day
+← A5 links forward to A6</t>
+        </is>
+      </c>
+      <c r="H33" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+Evaluate managed agent path</t>
+        </is>
+      </c>
+      <c r="I33" s="230" t="n">
+        <v>46147</v>
+      </c>
+      <c r="J33" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: compare managed vs self-hosted agents</t>
+        </is>
+      </c>
+      <c r="K33" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="211" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C34" s="212" t="inlineStr">
+        <is>
+          <t>Topview AI for Beginners: What to Test First Before You Commit to a Workflow</t>
+        </is>
+      </c>
+      <c r="D34" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E34" s="194" t="inlineStr">
+        <is>
+          <t>Guide  · 1,700 từ</t>
+        </is>
+      </c>
+      <c r="F34" s="194" t="inlineStr">
+        <is>
+          <t>topview ai for beginners</t>
+        </is>
+      </c>
+      <c r="G34" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, T3, /tools/topview-ai/
+← T1 links forward to T2</t>
+        </is>
+      </c>
+      <c r="H34" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Start with tool page</t>
+        </is>
+      </c>
+      <c r="I34" s="230" t="n">
+        <v>46148</v>
+      </c>
+      <c r="J34" s="213" t="inlineStr">
+        <is>
+          <t>Instructional · ToF-MoF
+Intent: reduce beginner friction</t>
+        </is>
+      </c>
+      <c r="K34" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="211" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="C35" s="212" t="inlineStr">
+        <is>
+          <t>Weekly AI Systems Roundup: Models, Agents, and Tool Moves Worth Tracking</t>
+        </is>
+      </c>
+      <c r="D35" s="193" t="inlineStr">
+        <is>
+          <t>Cluster N · News</t>
+        </is>
+      </c>
+      <c r="E35" s="194" t="inlineStr">
+        <is>
+          <t>Roundup  · 1,200 từ</t>
+        </is>
+      </c>
+      <c r="F35" s="194" t="inlineStr">
+        <is>
+          <t>weekly ai systems roundup</t>
+        </is>
+      </c>
+      <c r="G35" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, T1, /tools/
+← news summaries crosslink to current tools</t>
+        </is>
+      </c>
+      <c r="H35" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+Browse tools library</t>
+        </is>
+      </c>
+      <c r="I35" s="230" t="n">
+        <v>46149</v>
+      </c>
+      <c r="J35" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: stay current on AI systems</t>
+        </is>
+      </c>
+      <c r="K35" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="211" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="C36" s="212" t="inlineStr">
+        <is>
+          <t>Best Offer Page Type for Your Current Stage: Beginner Fit, Comparison, or Niche Path?</t>
+        </is>
+      </c>
+      <c r="D36" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E36" s="194" t="inlineStr">
+        <is>
+          <t>Decision Support  · 1,900 từ</t>
+        </is>
+      </c>
+      <c r="F36" s="194" t="inlineStr">
+        <is>
+          <t>best offer page type</t>
+        </is>
+      </c>
+      <c r="G36" s="213" t="inlineStr">
+        <is>
+          <t>→ O1, O3, /offers/find-your-best-affiliate-fit/
+← O1 links forward to O2</t>
+        </is>
+      </c>
+      <c r="H36" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Use best-fit offer page</t>
+        </is>
+      </c>
+      <c r="I36" s="230" t="n">
+        <v>46150</v>
+      </c>
+      <c r="J36" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: choose the right offer path</t>
+        </is>
+      </c>
+      <c r="K36" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="211" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C37" s="212" t="inlineStr">
+        <is>
+          <t>ConvertKit vs Beehiiv for AI Content Operators: Which One Fits Better?</t>
+        </is>
+      </c>
+      <c r="D37" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E37" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F37" s="194" t="inlineStr">
+        <is>
+          <t>convertkit vs beehiiv</t>
+        </is>
+      </c>
+      <c r="G37" s="213" t="inlineStr">
+        <is>
+          <t>→ P1, /programs/convertkit/, /programs/beehiiv/
+← P1 links to P2</t>
+        </is>
+      </c>
+      <c r="H37" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+View both program reviews</t>
+        </is>
+      </c>
+      <c r="I37" s="230" t="n">
+        <v>46151</v>
+      </c>
+      <c r="J37" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: choose email platform fit</t>
+        </is>
+      </c>
+      <c r="K37" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="211" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="C38" s="212" t="inlineStr">
+        <is>
+          <t>Best Use Cases for Abacus AI in Small Operator Teams</t>
+        </is>
+      </c>
+      <c r="D38" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E38" s="194" t="inlineStr">
+        <is>
+          <t>Use Case Guide  · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F38" s="194" t="inlineStr">
+        <is>
+          <t>abacus ai use cases</t>
+        </is>
+      </c>
+      <c r="G38" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, A10, /tools/abacus-ai/
+← A6 links across to A7</t>
+        </is>
+      </c>
+      <c r="H38" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See operator fit</t>
+        </is>
+      </c>
+      <c r="I38" s="230" t="n">
+        <v>46152</v>
+      </c>
+      <c r="J38" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: evaluate practical use cases</t>
+        </is>
+      </c>
+      <c r="K38" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="211" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C39" s="212" t="inlineStr">
+        <is>
+          <t>Best Use Cases for Topview AI in Affiliate and Ecommerce Creative Workflows</t>
+        </is>
+      </c>
+      <c r="D39" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E39" s="194" t="inlineStr">
+        <is>
+          <t>Use Case Guide  · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F39" s="194" t="inlineStr">
+        <is>
+          <t>topview ai use cases</t>
+        </is>
+      </c>
+      <c r="G39" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, T6, /tools/topview-ai/
+← T2 links forward to T3</t>
+        </is>
+      </c>
+      <c r="H39" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See creator workflow fit</t>
+        </is>
+      </c>
+      <c r="I39" s="230" t="n">
+        <v>46153</v>
+      </c>
+      <c r="J39" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: evaluate use cases for ads and ecommerce</t>
+        </is>
+      </c>
+      <c r="K39" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="211" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C40" s="212" t="inlineStr">
+        <is>
+          <t>Affiliate Program vs Affiliate Platform: What You Actually Need to Decide First</t>
+        </is>
+      </c>
+      <c r="D40" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E40" s="194" t="inlineStr">
+        <is>
+          <t>Explainer  · 1,900 từ</t>
+        </is>
+      </c>
+      <c r="F40" s="194" t="inlineStr">
+        <is>
+          <t>affiliate program vs affiliate platform</t>
+        </is>
+      </c>
+      <c r="G40" s="213" t="inlineStr">
+        <is>
+          <t>→ O1, O4, /offers/compare-affiliate-platforms/
+← O2 links forward to O3</t>
+        </is>
+      </c>
+      <c r="H40" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Compare affiliate platforms</t>
+        </is>
+      </c>
+      <c r="I40" s="230" t="n">
+        <v>46154</v>
+      </c>
+      <c r="J40" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: clarify decision order</t>
+        </is>
+      </c>
+      <c r="K40" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="211" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C41" s="212" t="inlineStr">
+        <is>
+          <t>n8n vs Make for Lean AI Operations: Which Automation Layer Fits Better?</t>
+        </is>
+      </c>
+      <c r="D41" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E41" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F41" s="194" t="inlineStr">
+        <is>
+          <t>n8n vs make</t>
+        </is>
+      </c>
+      <c r="G41" s="213" t="inlineStr">
+        <is>
+          <t>→ P1, /programs/n8n/, /programs/make/
+← workflow cluster links to P3</t>
+        </is>
+      </c>
+      <c r="H41" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+View automation program reviews</t>
+        </is>
+      </c>
+      <c r="I41" s="230" t="n">
+        <v>46155</v>
+      </c>
+      <c r="J41" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: choose automation layer</t>
+        </is>
+      </c>
+      <c r="K41" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="211" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="C42" s="212" t="inlineStr">
+        <is>
+          <t>Weekly AI Tool Signal Check: What Changed and What Actually Matters</t>
+        </is>
+      </c>
+      <c r="D42" s="193" t="inlineStr">
+        <is>
+          <t>Cluster N · News</t>
+        </is>
+      </c>
+      <c r="E42" s="194" t="inlineStr">
+        <is>
+          <t>Roundup  · 1,200 từ</t>
+        </is>
+      </c>
+      <c r="F42" s="194" t="inlineStr">
+        <is>
+          <t>weekly ai tool signal</t>
+        </is>
+      </c>
+      <c r="G42" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, A5, /search/
+← news links into search and tools</t>
+        </is>
+      </c>
+      <c r="H42" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+Search the content system</t>
+        </is>
+      </c>
+      <c r="I42" s="230" t="n">
+        <v>46156</v>
+      </c>
+      <c r="J42" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: interpret AI tool movement</t>
+        </is>
+      </c>
+      <c r="K42" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="211" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="C43" s="212" t="inlineStr">
+        <is>
+          <t>Abacus AI Model Stack Explained: When Multi-Model Access Is Actually Useful</t>
+        </is>
+      </c>
+      <c r="D43" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E43" s="194" t="inlineStr">
+        <is>
+          <t>Explainer  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F43" s="194" t="inlineStr">
+        <is>
+          <t>abacus ai model stack</t>
+        </is>
+      </c>
+      <c r="G43" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, A6, /tools/abacus-ai/
+← A5 links forward to A8</t>
+        </is>
+      </c>
+      <c r="H43" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Review Abacus AI model fit</t>
+        </is>
+      </c>
+      <c r="I43" s="230" t="n">
+        <v>46157</v>
+      </c>
+      <c r="J43" s="213" t="inlineStr">
+        <is>
+          <t>Informational · MoF
+Intent: understand multi-model value</t>
+        </is>
+      </c>
+      <c r="K43" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="211" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C44" s="212" t="inlineStr">
+        <is>
+          <t>Topview AI vs Higgsfield: Which Tool Fits Marketing Video Workflows Better?</t>
+        </is>
+      </c>
+      <c r="D44" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E44" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F44" s="194" t="inlineStr">
+        <is>
+          <t>topview ai vs higgsfield</t>
+        </is>
+      </c>
+      <c r="G44" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, /tools/topview-ai/, /tools/higgsfield/
+← T1 links forward to T4</t>
+        </is>
+      </c>
+      <c r="H44" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Choose the better tool fit</t>
+        </is>
+      </c>
+      <c r="I44" s="230" t="n">
+        <v>46158</v>
+      </c>
+      <c r="J44" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: compare visual workflow tools</t>
+        </is>
+      </c>
+      <c r="K44" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="211" t="inlineStr">
+        <is>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="C45" s="212" t="inlineStr">
+        <is>
+          <t>Best Affiliate Programs by Workflow Type, Not Just by Commission Size</t>
+        </is>
+      </c>
+      <c r="D45" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E45" s="194" t="inlineStr">
+        <is>
+          <t>Commercial Guide  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F45" s="194" t="inlineStr">
+        <is>
+          <t>best affiliate programs by workflow</t>
+        </is>
+      </c>
+      <c r="G45" s="213" t="inlineStr">
+        <is>
+          <t>→ O3, P1, /offers/affiliate-programs-by-niche/
+← O3 links forward to O4</t>
+        </is>
+      </c>
+      <c r="H45" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Browse programs by niche</t>
+        </is>
+      </c>
+      <c r="I45" s="230" t="n">
+        <v>46159</v>
+      </c>
+      <c r="J45" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: choose by workflow, not payout alone</t>
+        </is>
+      </c>
+      <c r="K45" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="211" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C46" s="212" t="inlineStr">
+        <is>
+          <t>Best AI Writing Tool for Program Reviews and Comparison Posts in 2026</t>
+        </is>
+      </c>
+      <c r="D46" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E46" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F46" s="194" t="inlineStr">
+        <is>
+          <t>best ai writing tool for reviews</t>
+        </is>
+      </c>
+      <c r="G46" s="213" t="inlineStr">
+        <is>
+          <t>→ P1, /programs/koala-writer/, /programs/writesonic/
+← comparison posts link to P4</t>
+        </is>
+      </c>
+      <c r="H46" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+View writing tool reviews</t>
+        </is>
+      </c>
+      <c r="I46" s="230" t="n">
+        <v>46160</v>
+      </c>
+      <c r="J46" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: pick a writing tool for monetized content</t>
+        </is>
+      </c>
+      <c r="K46" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="211" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="C47" s="212" t="inlineStr">
+        <is>
+          <t>How to Evaluate a Hosted Agent Platform Before Replacing Your Current Stack</t>
+        </is>
+      </c>
+      <c r="D47" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E47" s="194" t="inlineStr">
+        <is>
+          <t>Framework  · 1,900 từ</t>
+        </is>
+      </c>
+      <c r="F47" s="194" t="inlineStr">
+        <is>
+          <t>evaluate hosted agent platform</t>
+        </is>
+      </c>
+      <c r="G47" s="213" t="inlineStr">
+        <is>
+          <t>→ A6, A10, /tools/abacus-ai/
+← A6 links forward to A9</t>
+        </is>
+      </c>
+      <c r="H47" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+Evaluate managed platform fit</t>
+        </is>
+      </c>
+      <c r="I47" s="230" t="n">
+        <v>46161</v>
+      </c>
+      <c r="J47" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · BoF
+Intent: replacement evaluation</t>
+        </is>
+      </c>
+      <c r="K47" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="211" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C48" s="212" t="inlineStr">
+        <is>
+          <t>Topview AI Alternatives: When Another Visual Tool Is the Better Choice</t>
+        </is>
+      </c>
+      <c r="D48" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E48" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 1,800 từ</t>
+        </is>
+      </c>
+      <c r="F48" s="194" t="inlineStr">
+        <is>
+          <t>topview ai alternatives</t>
+        </is>
+      </c>
+      <c r="G48" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, T4, /tools/topview-ai/
+← T4 links forward to T5</t>
+        </is>
+      </c>
+      <c r="H48" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Review alternative tool paths</t>
+        </is>
+      </c>
+      <c r="I48" s="230" t="n">
+        <v>46162</v>
+      </c>
+      <c r="J48" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: evaluate alternatives</t>
+        </is>
+      </c>
+      <c r="K48" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="211" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C49" s="212" t="inlineStr">
+        <is>
+          <t>Weekly AI Market Analysis: Which Product Signals Are Real and Which Are Just Launch Noise?</t>
+        </is>
+      </c>
+      <c r="D49" s="193" t="inlineStr">
+        <is>
+          <t>Cluster N · News</t>
+        </is>
+      </c>
+      <c r="E49" s="194" t="inlineStr">
+        <is>
+          <t>Analysis  · 1,400 từ</t>
+        </is>
+      </c>
+      <c r="F49" s="194" t="inlineStr">
+        <is>
+          <t>weekly ai market analysis</t>
+        </is>
+      </c>
+      <c r="G49" s="213" t="inlineStr">
+        <is>
+          <t>→ N1, N2, /tools/
+← weekly analysis cluster links together</t>
+        </is>
+      </c>
+      <c r="H49" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+Browse tool pages</t>
+        </is>
+      </c>
+      <c r="I49" s="230" t="n">
+        <v>46163</v>
+      </c>
+      <c r="J49" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: interpret AI product signals</t>
+        </is>
+      </c>
+      <c r="K49" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="211" t="inlineStr">
+        <is>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C50" s="212" t="inlineStr">
+        <is>
+          <t>Recurring vs High-Ticket Offers in 2026: Which Route Fits Your Current System?</t>
+        </is>
+      </c>
+      <c r="D50" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E50" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F50" s="194" t="inlineStr">
+        <is>
+          <t>recurring vs high ticket offers</t>
+        </is>
+      </c>
+      <c r="G50" s="213" t="inlineStr">
+        <is>
+          <t>→ O2, /offers/recurring-commission-affiliate-programs/, /offers/high-ticket-affiliate-programs/
+← offer support posts link to O5</t>
+        </is>
+      </c>
+      <c r="H50" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+Compare offer models</t>
+        </is>
+      </c>
+      <c r="I50" s="230" t="n">
+        <v>46164</v>
+      </c>
+      <c r="J50" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: choose monetization model</t>
+        </is>
+      </c>
+      <c r="K50" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="211" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C51" s="212" t="inlineStr">
+        <is>
+          <t>Claude Pro vs ChatLLM Teams: Which Operator Layer Fits Better for Daily Work?</t>
+        </is>
+      </c>
+      <c r="D51" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E51" s="194" t="inlineStr">
+        <is>
+          <t>Comparison  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F51" s="194" t="inlineStr">
+        <is>
+          <t>claude pro vs chatllm teams</t>
+        </is>
+      </c>
+      <c r="G51" s="213" t="inlineStr">
+        <is>
+          <t>→ B0, A5, /programs/claude-pro/, /tools/abacus-ai/
+← workflow comparison posts link to P5</t>
+        </is>
+      </c>
+      <c r="H51" s="213" t="inlineStr">
+        <is>
+          <t>Strong CTA (BoF)
+Compare operator layers</t>
+        </is>
+      </c>
+      <c r="I51" s="230" t="n">
+        <v>46165</v>
+      </c>
+      <c r="J51" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF-BoF
+Intent: choose daily operator layer</t>
+        </is>
+      </c>
+      <c r="K51" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="211" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="C52" s="212" t="inlineStr">
+        <is>
+          <t>A Practical Abacus AI Workflow for Research, Writing, and Agent-Assisted Ops</t>
+        </is>
+      </c>
+      <c r="D52" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E52" s="194" t="inlineStr">
+        <is>
+          <t>Workflow  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F52" s="194" t="inlineStr">
+        <is>
+          <t>abacus ai workflow</t>
+        </is>
+      </c>
+      <c r="G52" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, P5, /tools/abacus-ai/
+← A7 and A9 link into A10</t>
+        </is>
+      </c>
+      <c r="H52" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See full workflow fit</t>
+        </is>
+      </c>
+      <c r="I52" s="230" t="n">
+        <v>46166</v>
+      </c>
+      <c r="J52" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: fit Abacus into a real workflow</t>
+        </is>
+      </c>
+      <c r="K52" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="211" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C53" s="212" t="inlineStr">
+        <is>
+          <t>How to Use Topview AI for Affiliate Product Videos Without Overbuilding the Stack</t>
+        </is>
+      </c>
+      <c r="D53" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E53" s="194" t="inlineStr">
+        <is>
+          <t>How-to  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F53" s="194" t="inlineStr">
+        <is>
+          <t>how to use topview ai</t>
+        </is>
+      </c>
+      <c r="G53" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, P1, /tools/topview-ai/
+← T3 links forward to T6</t>
+        </is>
+      </c>
+      <c r="H53" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF/BoF)
+Use Topview in a real stack</t>
+        </is>
+      </c>
+      <c r="I53" s="230" t="n">
+        <v>46167</v>
+      </c>
+      <c r="J53" s="213" t="inlineStr">
+        <is>
+          <t>Instructional · MoF-BoF
+Intent: apply Topview in affiliate workflows</t>
+        </is>
+      </c>
+      <c r="K53" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="211" t="inlineStr">
+        <is>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="C54" s="212" t="inlineStr">
+        <is>
+          <t>The Fastest Way to Find Your Best Affiliate Fit Without Starting Over Repeatedly</t>
+        </is>
+      </c>
+      <c r="D54" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E54" s="194" t="inlineStr">
+        <is>
+          <t>Decision Support  · 1,900 từ</t>
+        </is>
+      </c>
+      <c r="F54" s="194" t="inlineStr">
+        <is>
+          <t>find your best affiliate fit fast</t>
+        </is>
+      </c>
+      <c r="G54" s="213" t="inlineStr">
+        <is>
+          <t>→ O1, /offers/find-your-best-affiliate-fit/
+← O1/O2 support O6</t>
+        </is>
+      </c>
+      <c r="H54" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Use the best-fit page</t>
+        </is>
+      </c>
+      <c r="I54" s="230" t="n">
+        <v>46168</v>
+      </c>
+      <c r="J54" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: reduce repeated restart cycles</t>
+        </is>
+      </c>
+      <c r="K54" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="211" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="C55" s="212" t="inlineStr">
+        <is>
+          <t>Best AI Tools for Landing Pages, Funnels, and Conversion Assets in 2026</t>
+        </is>
+      </c>
+      <c r="D55" s="193" t="inlineStr">
+        <is>
+          <t>Cluster P · Programs &amp; Workflow</t>
+        </is>
+      </c>
+      <c r="E55" s="194" t="inlineStr">
+        <is>
+          <t>Commercial Guide  · 2,100 từ</t>
+        </is>
+      </c>
+      <c r="F55" s="194" t="inlineStr">
+        <is>
+          <t>best ai tools for landing pages</t>
+        </is>
+      </c>
+      <c r="G55" s="213" t="inlineStr">
+        <is>
+          <t>→ P1, /tools/, /offers/affiliate-tools-for-content-creators/
+← program/workflow support posts link to P6</t>
+        </is>
+      </c>
+      <c r="H55" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+See creator tools and conversion paths</t>
+        </is>
+      </c>
+      <c r="I55" s="230" t="n">
+        <v>46169</v>
+      </c>
+      <c r="J55" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: choose tools for landing and funnel work</t>
+        </is>
+      </c>
+      <c r="K55" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="211" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C56" s="212" t="inlineStr">
+        <is>
+          <t>Weekly AI Systems Roundup: Agent Products, Creator Tools, and Search Shifts</t>
+        </is>
+      </c>
+      <c r="D56" s="193" t="inlineStr">
+        <is>
+          <t>Cluster N · News</t>
+        </is>
+      </c>
+      <c r="E56" s="194" t="inlineStr">
+        <is>
+          <t>Roundup  · 1,200 từ</t>
+        </is>
+      </c>
+      <c r="F56" s="194" t="inlineStr">
+        <is>
+          <t>weekly ai systems roundup may</t>
+        </is>
+      </c>
+      <c r="G56" s="213" t="inlineStr">
+        <is>
+          <t>→ N1, N2, /search/, /tools/
+← weekly news chain</t>
+        </is>
+      </c>
+      <c r="H56" s="213" t="inlineStr">
+        <is>
+          <t>Soft CTA (ToF)
+Search the latest system content</t>
+        </is>
+      </c>
+      <c r="I56" s="230" t="n">
+        <v>46170</v>
+      </c>
+      <c r="J56" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF
+Intent: stay current across AI systems</t>
+        </is>
+      </c>
+      <c r="K56" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="211" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="C57" s="212" t="inlineStr">
+        <is>
+          <t>Abacus AI for Non-Developers: Where It Helps and Where It Is Overkill</t>
+        </is>
+      </c>
+      <c r="D57" s="193" t="inlineStr">
+        <is>
+          <t>Cluster A · Abacus AI</t>
+        </is>
+      </c>
+      <c r="E57" s="194" t="inlineStr">
+        <is>
+          <t>Guide  · 1,900 từ</t>
+        </is>
+      </c>
+      <c r="F57" s="194" t="inlineStr">
+        <is>
+          <t>abacus ai for non developers</t>
+        </is>
+      </c>
+      <c r="G57" s="213" t="inlineStr">
+        <is>
+          <t>→ A5, A10, /tools/abacus-ai/
+← A5 links forward to A11</t>
+        </is>
+      </c>
+      <c r="H57" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Review non-developer fit</t>
+        </is>
+      </c>
+      <c r="I57" s="230" t="n">
+        <v>46171</v>
+      </c>
+      <c r="J57" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: evaluate accessibility and scope</t>
+        </is>
+      </c>
+      <c r="K57" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="211" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C58" s="212" t="inlineStr">
+        <is>
+          <t>A Creator Workflow Using Topview AI, Claude, and Automation Tools</t>
+        </is>
+      </c>
+      <c r="D58" s="193" t="inlineStr">
+        <is>
+          <t>Cluster T · Topview AI</t>
+        </is>
+      </c>
+      <c r="E58" s="194" t="inlineStr">
+        <is>
+          <t>Workflow  · 2,200 từ</t>
+        </is>
+      </c>
+      <c r="F58" s="194" t="inlineStr">
+        <is>
+          <t>topview ai workflow</t>
+        </is>
+      </c>
+      <c r="G58" s="213" t="inlineStr">
+        <is>
+          <t>→ T1, B0, /tools/topview-ai/
+← T6 links forward to T7</t>
+        </is>
+      </c>
+      <c r="H58" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Go from tool to workflow</t>
+        </is>
+      </c>
+      <c r="I58" s="230" t="n">
+        <v>46172</v>
+      </c>
+      <c r="J58" s="213" t="inlineStr">
+        <is>
+          <t>Commercial · MoF
+Intent: fit Topview into a wider system</t>
+        </is>
+      </c>
+      <c r="K58" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="211" t="inlineStr">
+        <is>
+          <t>O7</t>
+        </is>
+      </c>
+      <c r="C59" s="212" t="inlineStr">
+        <is>
+          <t>Programs, Tools, and Offers: How the MoltyFlywheel System Fits Together in Practice</t>
+        </is>
+      </c>
+      <c r="D59" s="193" t="inlineStr">
+        <is>
+          <t>Cluster O · Decision Support</t>
+        </is>
+      </c>
+      <c r="E59" s="194" t="inlineStr">
+        <is>
+          <t>System Guide  · 2,000 từ</t>
+        </is>
+      </c>
+      <c r="F59" s="194" t="inlineStr">
+        <is>
+          <t>programs tools offers system</t>
+        </is>
+      </c>
+      <c r="G59" s="213" t="inlineStr">
+        <is>
+          <t>→ O1, /tools/, /programs/, /offers/
+← route-support cluster links back to O7</t>
+        </is>
+      </c>
+      <c r="H59" s="213" t="inlineStr">
+        <is>
+          <t>Medium CTA (MoF)
+Use the full MoltyFlywheel system</t>
+        </is>
+      </c>
+      <c r="I59" s="230" t="n">
+        <v>46173</v>
+      </c>
+      <c r="J59" s="213" t="inlineStr">
+        <is>
+          <t>Informational · ToF-MoF
+Intent: understand how the site system connects</t>
+        </is>
+      </c>
+      <c r="K59" s="214" t="inlineStr">
+        <is>
+          <t>⬜ Chưa viết</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish April 27 Agentic AI workforce post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -434,7 +434,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="231">
+  <cellXfs count="232">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1124,6 +1124,7 @@
     <xf numFmtId="164" fontId="16" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2649,32 +2650,32 @@
           <t>W5</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="114" t="inlineStr">
         <is>
           <t>T6, 01/05</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="114" t="inlineStr">
         <is>
           <t>A5 — What Is Abacus AI? A Practical Guide to Models, Agents, and the Managed Claw Path</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="114" t="inlineStr">
         <is>
           <t>Track A · Abacus AI</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="114" t="inlineStr">
         <is>
           <t>Guide (~2,000 từ)</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="114" t="inlineStr">
         <is>
           <t>ToF/MoF</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="114" t="inlineStr">
         <is>
           <t>🔥 Hot</t>
         </is>
@@ -3692,6 +3693,12 @@
           <t>Ghi chú: Queue tháng 4 đã được port và tháng 5 đã được lên kế hoạch daily cadence 1 bài/ngày. Các bài tháng 5 hiện ở trạng thái planned và chưa viết trừ khi có task sản xuất riêng.</t>
         </is>
       </c>
+      <c r="C62" s="140" t="n"/>
+      <c r="D62" s="140" t="n"/>
+      <c r="E62" s="140" t="n"/>
+      <c r="F62" s="140" t="n"/>
+      <c r="G62" s="140" t="n"/>
+      <c r="H62" s="231" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4057,7 +4064,7 @@
       </c>
       <c r="K9" s="202" t="inlineStr">
         <is>
-          <t>🟡 Đã viết / chờ đăng</t>
+          <t>✅ Đã đăng (27/04)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish May 1 Abacus AI post
</commit_message>
<xml_diff>
--- a/docs/lich_xuat_ban_moltyflywheel.xlsx
+++ b/docs/lich_xuat_ban_moltyflywheel.xlsx
@@ -3717,7 +3717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:K59"/>
+  <dimension ref="A2:K59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="114" min="1" max="1"/>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K29" s="214" t="inlineStr">
         <is>
-          <t>⬜ Chưa viết</t>
+          <t>✅ Đã đăng (01/05)</t>
         </is>
       </c>
     </row>

</xml_diff>